<commit_message>
Continuacion/ mejora de motodos y preguntar (s/n)
</commit_message>
<xml_diff>
--- a/myapp/src/main/resources/Listado_Obra_A.xlsx
+++ b/myapp/src/main/resources/Listado_Obra_A.xlsx
@@ -3,12 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\App_TecnoMat\app_lectorArchivos\myapp\src\main\resources\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6433628C-52F4-4AF5-83FC-69306858B642}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{1D1C93DB-C31D-4158-BF75-6A7B962B5151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,6 +14,7 @@
     <externalReference r:id="rId2"/>
   </externalReferences>
   <calcPr calcId="191029"/>
+  <oleSize ref="A1"/>
 </workbook>
 </file>
 
@@ -468,9 +464,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -506,33 +499,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -550,12 +516,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -566,6 +526,42 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1003,87 +999,87 @@
       </c>
       <c r="B2" s="7"/>
       <c r="C2" s="7"/>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="36" t="s">
         <v>57</v>
       </c>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
+      <c r="G2" s="36"/>
       <c r="H2" s="7"/>
       <c r="I2" s="7"/>
-      <c r="J2" s="9"/>
+      <c r="J2" s="8"/>
     </row>
     <row r="3" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="7"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="12"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="11"/>
       <c r="F3" s="7"/>
-      <c r="G3" s="13"/>
+      <c r="G3" s="12"/>
       <c r="H3" s="7"/>
       <c r="I3" s="7"/>
-      <c r="J3" s="14"/>
+      <c r="J3" s="13"/>
     </row>
     <row r="4" spans="1:10" ht="18" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>1</v>
       </c>
       <c r="B4" s="7"/>
-      <c r="C4" s="15" t="s">
+      <c r="C4" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="16" t="s">
+      <c r="D4" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="E4" s="17"/>
+      <c r="E4" s="16"/>
       <c r="F4" s="7"/>
       <c r="G4" s="7"/>
       <c r="H4" s="7"/>
-      <c r="I4" s="18"/>
-      <c r="J4" s="19"/>
+      <c r="I4" s="17"/>
+      <c r="J4" s="18"/>
     </row>
     <row r="5" spans="1:10" ht="54" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>1</v>
       </c>
       <c r="B5" s="7"/>
-      <c r="C5" s="15" t="s">
+      <c r="C5" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="20" t="s">
+      <c r="D5" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="E5" s="21"/>
+      <c r="E5" s="20"/>
       <c r="F5" s="7"/>
-      <c r="G5" s="22" t="s">
+      <c r="G5" s="37" t="s">
         <v>4</v>
       </c>
-      <c r="H5" s="22"/>
-      <c r="I5" s="23" t="s">
+      <c r="H5" s="37"/>
+      <c r="I5" s="38" t="s">
         <v>60</v>
       </c>
-      <c r="J5" s="24"/>
+      <c r="J5" s="39"/>
     </row>
     <row r="6" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>1</v>
       </c>
       <c r="B6" s="7"/>
-      <c r="C6" s="15" t="s">
+      <c r="C6" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="25" t="s">
+      <c r="D6" s="40" t="s">
         <v>59</v>
       </c>
-      <c r="E6" s="26"/>
+      <c r="E6" s="41"/>
       <c r="F6" s="7"/>
-      <c r="G6" s="27" t="s">
+      <c r="G6" s="42" t="s">
         <v>6</v>
       </c>
-      <c r="H6" s="27"/>
+      <c r="H6" s="42"/>
       <c r="I6" s="43">
         <v>46449</v>
       </c>
@@ -1096,929 +1092,929 @@
       <c r="D7" s="7"/>
       <c r="E7" s="7"/>
       <c r="F7" s="7"/>
-      <c r="G7" s="30" t="s">
+      <c r="G7" s="31" t="s">
         <v>7</v>
       </c>
-      <c r="H7" s="30"/>
-      <c r="I7" s="28">
+      <c r="H7" s="31"/>
+      <c r="I7" s="32">
         <v>46111</v>
       </c>
-      <c r="J7" s="29"/>
+      <c r="J7" s="33"/>
     </row>
     <row r="8" spans="1:10" ht="18" x14ac:dyDescent="0.25">
-      <c r="A8" s="31" t="s">
+      <c r="A8" s="21" t="s">
         <v>1</v>
       </c>
       <c r="B8" s="7"/>
-      <c r="C8" s="32"/>
-      <c r="D8" s="32"/>
-      <c r="E8" s="33"/>
-      <c r="F8" s="34"/>
-      <c r="G8" s="34"/>
-      <c r="H8" s="34"/>
-      <c r="I8" s="34"/>
-      <c r="J8" s="35"/>
+      <c r="C8" s="22"/>
+      <c r="D8" s="22"/>
+      <c r="E8" s="23"/>
+      <c r="F8" s="24"/>
+      <c r="G8" s="24"/>
+      <c r="H8" s="24"/>
+      <c r="I8" s="24"/>
+      <c r="J8" s="25"/>
     </row>
     <row r="9" spans="1:10" ht="24" x14ac:dyDescent="0.25">
-      <c r="A9" s="36" t="s">
+      <c r="A9" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B9" s="36" t="s">
+      <c r="B9" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="C9" s="36" t="s">
+      <c r="C9" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="D9" s="36" t="s">
+      <c r="D9" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="E9" s="37" t="s">
+      <c r="E9" s="34" t="s">
         <v>11</v>
       </c>
-      <c r="F9" s="38"/>
-      <c r="G9" s="37" t="s">
+      <c r="F9" s="35"/>
+      <c r="G9" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="H9" s="38"/>
-      <c r="I9" s="39" t="s">
+      <c r="H9" s="35"/>
+      <c r="I9" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="J9" s="36" t="s">
+      <c r="J9" s="26" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" s="40">
+      <c r="A10" s="28">
         <v>76666</v>
       </c>
-      <c r="B10" s="40" t="s">
+      <c r="B10" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="40" t="s">
+      <c r="C10" s="28" t="s">
         <v>16</v>
       </c>
-      <c r="D10" s="41" t="s">
+      <c r="D10" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="E10" s="42">
-        <v>1</v>
-      </c>
-      <c r="F10" s="40"/>
-      <c r="G10" s="40"/>
-      <c r="H10" s="40"/>
-      <c r="I10" s="40">
+      <c r="E10" s="30">
+        <v>1</v>
+      </c>
+      <c r="F10" s="28"/>
+      <c r="G10" s="28"/>
+      <c r="H10" s="28"/>
+      <c r="I10" s="28">
         <f>E10*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J10" s="41"/>
+      <c r="J10" s="29"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11" s="40">
+      <c r="A11" s="28">
         <v>76665</v>
       </c>
-      <c r="B11" s="40" t="s">
+      <c r="B11" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="40" t="s">
+      <c r="C11" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="D11" s="41" t="s">
+      <c r="D11" s="29" t="s">
         <v>19</v>
       </c>
-      <c r="E11" s="42">
-        <v>1</v>
-      </c>
-      <c r="F11" s="40"/>
-      <c r="G11" s="40"/>
-      <c r="H11" s="40"/>
-      <c r="I11" s="40">
+      <c r="E11" s="30">
+        <v>1</v>
+      </c>
+      <c r="F11" s="28"/>
+      <c r="G11" s="28"/>
+      <c r="H11" s="28"/>
+      <c r="I11" s="28">
         <f>E11*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J11" s="41"/>
+      <c r="J11" s="29"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12" s="40">
+      <c r="A12" s="28">
         <v>75884</v>
       </c>
-      <c r="B12" s="40" t="s">
+      <c r="B12" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="C12" s="40">
+      <c r="C12" s="28">
         <v>607287</v>
       </c>
-      <c r="D12" s="41" t="s">
+      <c r="D12" s="29" t="s">
         <v>20</v>
       </c>
-      <c r="E12" s="42">
-        <v>1</v>
-      </c>
-      <c r="F12" s="40"/>
-      <c r="G12" s="40"/>
-      <c r="H12" s="40"/>
-      <c r="I12" s="40">
+      <c r="E12" s="30">
+        <v>1</v>
+      </c>
+      <c r="F12" s="28"/>
+      <c r="G12" s="28"/>
+      <c r="H12" s="28"/>
+      <c r="I12" s="28">
         <f>E12*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J12" s="41"/>
+      <c r="J12" s="29"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A13" s="40">
+      <c r="A13" s="28">
         <v>73809</v>
       </c>
-      <c r="B13" s="40" t="s">
+      <c r="B13" s="28" t="s">
         <v>21</v>
       </c>
-      <c r="C13" s="40">
+      <c r="C13" s="28">
         <v>534017</v>
       </c>
-      <c r="D13" s="41" t="s">
+      <c r="D13" s="29" t="s">
         <v>22</v>
       </c>
-      <c r="E13" s="42">
+      <c r="E13" s="30">
         <v>4</v>
       </c>
-      <c r="F13" s="40"/>
-      <c r="G13" s="40"/>
-      <c r="H13" s="40"/>
-      <c r="I13" s="40">
+      <c r="F13" s="28"/>
+      <c r="G13" s="28"/>
+      <c r="H13" s="28"/>
+      <c r="I13" s="28">
         <f>E13*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>4</v>
       </c>
-      <c r="J13" s="41"/>
+      <c r="J13" s="29"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A14" s="40">
+      <c r="A14" s="28">
         <v>65794</v>
       </c>
-      <c r="B14" s="40" t="s">
+      <c r="B14" s="28" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="40">
+      <c r="C14" s="28">
         <v>550290</v>
       </c>
-      <c r="D14" s="41" t="s">
+      <c r="D14" s="29" t="s">
         <v>23</v>
       </c>
-      <c r="E14" s="42">
-        <v>1</v>
-      </c>
-      <c r="F14" s="40"/>
-      <c r="G14" s="40"/>
-      <c r="H14" s="40"/>
-      <c r="I14" s="40">
+      <c r="E14" s="30">
+        <v>1</v>
+      </c>
+      <c r="F14" s="28"/>
+      <c r="G14" s="28"/>
+      <c r="H14" s="28"/>
+      <c r="I14" s="28">
         <f>E14*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J14" s="41"/>
+      <c r="J14" s="29"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A15" s="40"/>
-      <c r="B15" s="40" t="s">
-        <v>24</v>
-      </c>
-      <c r="C15" s="40" t="s">
+      <c r="A15" s="28"/>
+      <c r="B15" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C15" s="28" t="s">
         <v>25</v>
       </c>
-      <c r="D15" s="41" t="s">
+      <c r="D15" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="E15" s="42">
-        <v>1</v>
-      </c>
-      <c r="F15" s="40"/>
-      <c r="G15" s="40"/>
-      <c r="H15" s="40"/>
-      <c r="I15" s="40">
+      <c r="E15" s="30">
+        <v>1</v>
+      </c>
+      <c r="F15" s="28"/>
+      <c r="G15" s="28"/>
+      <c r="H15" s="28"/>
+      <c r="I15" s="28">
         <f>E15*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J15" s="41"/>
+      <c r="J15" s="29"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A16" s="40">
+      <c r="A16" s="28">
         <v>79562</v>
       </c>
-      <c r="B16" s="40" t="s">
-        <v>24</v>
-      </c>
-      <c r="C16" s="40">
+      <c r="B16" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C16" s="28">
         <v>5818</v>
       </c>
-      <c r="D16" s="41" t="s">
+      <c r="D16" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="E16" s="42">
+      <c r="E16" s="30">
         <v>4</v>
       </c>
-      <c r="F16" s="40"/>
-      <c r="G16" s="40"/>
-      <c r="H16" s="40"/>
-      <c r="I16" s="40">
+      <c r="F16" s="28"/>
+      <c r="G16" s="28"/>
+      <c r="H16" s="28"/>
+      <c r="I16" s="28">
         <f>E16*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>4</v>
       </c>
-      <c r="J16" s="41"/>
+      <c r="J16" s="29"/>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A17" s="40">
+      <c r="A17" s="28">
         <v>79563</v>
       </c>
-      <c r="B17" s="40" t="s">
-        <v>24</v>
-      </c>
-      <c r="C17" s="40">
+      <c r="B17" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C17" s="28">
         <v>13302</v>
       </c>
-      <c r="D17" s="41" t="s">
+      <c r="D17" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="E17" s="42">
+      <c r="E17" s="30">
         <v>4</v>
       </c>
-      <c r="F17" s="40"/>
-      <c r="G17" s="40"/>
-      <c r="H17" s="40"/>
-      <c r="I17" s="40">
+      <c r="F17" s="28"/>
+      <c r="G17" s="28"/>
+      <c r="H17" s="28"/>
+      <c r="I17" s="28">
         <f>E17*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>4</v>
       </c>
-      <c r="J17" s="41"/>
+      <c r="J17" s="29"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A18" s="40">
+      <c r="A18" s="28">
         <v>79564</v>
       </c>
-      <c r="B18" s="40" t="s">
-        <v>24</v>
-      </c>
-      <c r="C18" s="40">
+      <c r="B18" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C18" s="28">
         <v>20051</v>
       </c>
-      <c r="D18" s="41" t="s">
+      <c r="D18" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="E18" s="42">
+      <c r="E18" s="30">
         <v>3</v>
       </c>
-      <c r="F18" s="40"/>
-      <c r="G18" s="40"/>
-      <c r="H18" s="40"/>
-      <c r="I18" s="40">
+      <c r="F18" s="28"/>
+      <c r="G18" s="28"/>
+      <c r="H18" s="28"/>
+      <c r="I18" s="28">
         <f>E18*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>3</v>
       </c>
-      <c r="J18" s="41"/>
+      <c r="J18" s="29"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A19" s="40">
+      <c r="A19" s="28">
         <v>71109</v>
       </c>
-      <c r="B19" s="40" t="s">
-        <v>24</v>
-      </c>
-      <c r="C19" s="40">
+      <c r="B19" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C19" s="28">
         <v>20119</v>
       </c>
-      <c r="D19" s="41" t="s">
+      <c r="D19" s="29" t="s">
         <v>30</v>
       </c>
-      <c r="E19" s="42">
-        <v>1</v>
-      </c>
-      <c r="F19" s="40"/>
-      <c r="G19" s="40"/>
-      <c r="H19" s="40"/>
-      <c r="I19" s="40">
+      <c r="E19" s="30">
+        <v>1</v>
+      </c>
+      <c r="F19" s="28"/>
+      <c r="G19" s="28"/>
+      <c r="H19" s="28"/>
+      <c r="I19" s="28">
         <f>E19*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J19" s="41"/>
+      <c r="J19" s="29"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A20" s="40">
+      <c r="A20" s="28">
         <v>80696</v>
       </c>
-      <c r="B20" s="40" t="s">
-        <v>24</v>
-      </c>
-      <c r="C20" s="40">
+      <c r="B20" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C20" s="28">
         <v>20139</v>
       </c>
-      <c r="D20" s="41" t="s">
+      <c r="D20" s="29" t="s">
         <v>31</v>
       </c>
-      <c r="E20" s="42">
-        <v>1</v>
-      </c>
-      <c r="F20" s="40"/>
-      <c r="G20" s="40"/>
-      <c r="H20" s="40"/>
-      <c r="I20" s="40">
+      <c r="E20" s="30">
+        <v>1</v>
+      </c>
+      <c r="F20" s="28"/>
+      <c r="G20" s="28"/>
+      <c r="H20" s="28"/>
+      <c r="I20" s="28">
         <f>E20*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J20" s="41"/>
+      <c r="J20" s="29"/>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A21" s="40">
+      <c r="A21" s="28">
         <v>80697</v>
       </c>
-      <c r="B21" s="40" t="s">
-        <v>24</v>
-      </c>
-      <c r="C21" s="40">
+      <c r="B21" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C21" s="28">
         <v>20149</v>
       </c>
-      <c r="D21" s="41" t="s">
+      <c r="D21" s="29" t="s">
         <v>32</v>
       </c>
-      <c r="E21" s="42">
-        <v>1</v>
-      </c>
-      <c r="F21" s="40"/>
-      <c r="G21" s="40"/>
-      <c r="H21" s="40"/>
-      <c r="I21" s="40">
+      <c r="E21" s="30">
+        <v>1</v>
+      </c>
+      <c r="F21" s="28"/>
+      <c r="G21" s="28"/>
+      <c r="H21" s="28"/>
+      <c r="I21" s="28">
         <f>E21*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J21" s="41"/>
+      <c r="J21" s="29"/>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A22" s="40">
+      <c r="A22" s="28">
         <v>80698</v>
       </c>
-      <c r="B22" s="40" t="s">
-        <v>24</v>
-      </c>
-      <c r="C22" s="40">
+      <c r="B22" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C22" s="28">
         <v>20169</v>
       </c>
-      <c r="D22" s="41" t="s">
+      <c r="D22" s="29" t="s">
         <v>33</v>
       </c>
-      <c r="E22" s="42">
-        <v>1</v>
-      </c>
-      <c r="F22" s="40"/>
-      <c r="G22" s="40"/>
-      <c r="H22" s="40"/>
-      <c r="I22" s="40">
+      <c r="E22" s="30">
+        <v>1</v>
+      </c>
+      <c r="F22" s="28"/>
+      <c r="G22" s="28"/>
+      <c r="H22" s="28"/>
+      <c r="I22" s="28">
         <f>E22*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J22" s="41"/>
+      <c r="J22" s="29"/>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A23" s="40">
+      <c r="A23" s="28">
         <v>79672</v>
       </c>
-      <c r="B23" s="40" t="s">
-        <v>24</v>
-      </c>
-      <c r="C23" s="40">
+      <c r="B23" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C23" s="28">
         <v>20201</v>
       </c>
-      <c r="D23" s="41" t="s">
+      <c r="D23" s="29" t="s">
         <v>34</v>
       </c>
-      <c r="E23" s="42">
+      <c r="E23" s="30">
         <v>2</v>
       </c>
-      <c r="F23" s="40"/>
-      <c r="G23" s="40"/>
-      <c r="H23" s="40"/>
-      <c r="I23" s="40">
+      <c r="F23" s="28"/>
+      <c r="G23" s="28"/>
+      <c r="H23" s="28"/>
+      <c r="I23" s="28">
         <f>E23*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>2</v>
       </c>
-      <c r="J23" s="41"/>
+      <c r="J23" s="29"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A24" s="40">
+      <c r="A24" s="28">
         <v>80699</v>
       </c>
-      <c r="B24" s="40" t="s">
-        <v>24</v>
-      </c>
-      <c r="C24" s="40">
+      <c r="B24" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C24" s="28">
         <v>20204</v>
       </c>
-      <c r="D24" s="41" t="s">
+      <c r="D24" s="29" t="s">
         <v>35</v>
       </c>
-      <c r="E24" s="42">
-        <v>1</v>
-      </c>
-      <c r="F24" s="40"/>
-      <c r="G24" s="40"/>
-      <c r="H24" s="40"/>
-      <c r="I24" s="40">
+      <c r="E24" s="30">
+        <v>1</v>
+      </c>
+      <c r="F24" s="28"/>
+      <c r="G24" s="28"/>
+      <c r="H24" s="28"/>
+      <c r="I24" s="28">
         <f>E24*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J24" s="41"/>
+      <c r="J24" s="29"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A25" s="40">
+      <c r="A25" s="28">
         <v>80700</v>
       </c>
-      <c r="B25" s="40" t="s">
-        <v>24</v>
-      </c>
-      <c r="C25" s="40">
+      <c r="B25" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C25" s="28">
         <v>20207</v>
       </c>
-      <c r="D25" s="41" t="s">
+      <c r="D25" s="29" t="s">
         <v>36</v>
       </c>
-      <c r="E25" s="42">
-        <v>1</v>
-      </c>
-      <c r="F25" s="40"/>
-      <c r="G25" s="40"/>
-      <c r="H25" s="40"/>
-      <c r="I25" s="40">
+      <c r="E25" s="30">
+        <v>1</v>
+      </c>
+      <c r="F25" s="28"/>
+      <c r="G25" s="28"/>
+      <c r="H25" s="28"/>
+      <c r="I25" s="28">
         <f>E25*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J25" s="41"/>
+      <c r="J25" s="29"/>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A26" s="40">
+      <c r="A26" s="28">
         <v>80701</v>
       </c>
-      <c r="B26" s="40" t="s">
-        <v>24</v>
-      </c>
-      <c r="C26" s="40">
+      <c r="B26" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C26" s="28">
         <v>20211</v>
       </c>
-      <c r="D26" s="41" t="s">
+      <c r="D26" s="29" t="s">
         <v>37</v>
       </c>
-      <c r="E26" s="42">
+      <c r="E26" s="30">
         <v>2</v>
       </c>
-      <c r="F26" s="40"/>
-      <c r="G26" s="40"/>
-      <c r="H26" s="40"/>
-      <c r="I26" s="40">
+      <c r="F26" s="28"/>
+      <c r="G26" s="28"/>
+      <c r="H26" s="28"/>
+      <c r="I26" s="28">
         <f>E26*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>2</v>
       </c>
-      <c r="J26" s="41"/>
+      <c r="J26" s="29"/>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A27" s="40">
+      <c r="A27" s="28">
         <v>80702</v>
       </c>
-      <c r="B27" s="40" t="s">
-        <v>24</v>
-      </c>
-      <c r="C27" s="40">
+      <c r="B27" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C27" s="28">
         <v>20279</v>
       </c>
-      <c r="D27" s="41" t="s">
+      <c r="D27" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="E27" s="42">
-        <v>1</v>
-      </c>
-      <c r="F27" s="40"/>
-      <c r="G27" s="40"/>
-      <c r="H27" s="40"/>
-      <c r="I27" s="40">
+      <c r="E27" s="30">
+        <v>1</v>
+      </c>
+      <c r="F27" s="28"/>
+      <c r="G27" s="28"/>
+      <c r="H27" s="28"/>
+      <c r="I27" s="28">
         <f>E27*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J27" s="41"/>
+      <c r="J27" s="29"/>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A28" s="40">
+      <c r="A28" s="28">
         <v>79565</v>
       </c>
-      <c r="B28" s="40" t="s">
-        <v>24</v>
-      </c>
-      <c r="C28" s="40">
+      <c r="B28" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C28" s="28">
         <v>20291</v>
       </c>
-      <c r="D28" s="41" t="s">
+      <c r="D28" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="E28" s="42">
+      <c r="E28" s="30">
         <v>2</v>
       </c>
-      <c r="F28" s="40"/>
-      <c r="G28" s="40"/>
-      <c r="H28" s="40"/>
-      <c r="I28" s="40">
+      <c r="F28" s="28"/>
+      <c r="G28" s="28"/>
+      <c r="H28" s="28"/>
+      <c r="I28" s="28">
         <f>E28*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>2</v>
       </c>
-      <c r="J28" s="41"/>
+      <c r="J28" s="29"/>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A29" s="40">
+      <c r="A29" s="28">
         <v>79671</v>
       </c>
-      <c r="B29" s="40" t="s">
-        <v>24</v>
-      </c>
-      <c r="C29" s="40">
+      <c r="B29" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C29" s="28">
         <v>20300</v>
       </c>
-      <c r="D29" s="41" t="s">
+      <c r="D29" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="E29" s="42">
+      <c r="E29" s="30">
         <v>2</v>
       </c>
-      <c r="F29" s="40"/>
-      <c r="G29" s="40"/>
-      <c r="H29" s="40"/>
-      <c r="I29" s="40">
+      <c r="F29" s="28"/>
+      <c r="G29" s="28"/>
+      <c r="H29" s="28"/>
+      <c r="I29" s="28">
         <f>E29*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>2</v>
       </c>
-      <c r="J29" s="41"/>
+      <c r="J29" s="29"/>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A30" s="40">
+      <c r="A30" s="28">
         <v>80703</v>
       </c>
-      <c r="B30" s="40" t="s">
-        <v>24</v>
-      </c>
-      <c r="C30" s="40">
+      <c r="B30" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C30" s="28">
         <v>20307</v>
       </c>
-      <c r="D30" s="41" t="s">
+      <c r="D30" s="29" t="s">
         <v>41</v>
       </c>
-      <c r="E30" s="42">
-        <v>1</v>
-      </c>
-      <c r="F30" s="40"/>
-      <c r="G30" s="40"/>
-      <c r="H30" s="40"/>
-      <c r="I30" s="40">
+      <c r="E30" s="30">
+        <v>1</v>
+      </c>
+      <c r="F30" s="28"/>
+      <c r="G30" s="28"/>
+      <c r="H30" s="28"/>
+      <c r="I30" s="28">
         <f>E30*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J30" s="41"/>
+      <c r="J30" s="29"/>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A31" s="40">
+      <c r="A31" s="28">
         <v>80704</v>
       </c>
-      <c r="B31" s="40" t="s">
-        <v>24</v>
-      </c>
-      <c r="C31" s="40">
+      <c r="B31" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C31" s="28">
         <v>20310</v>
       </c>
-      <c r="D31" s="41" t="s">
+      <c r="D31" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="E31" s="42">
+      <c r="E31" s="30">
         <v>2</v>
       </c>
-      <c r="F31" s="40"/>
-      <c r="G31" s="40"/>
-      <c r="H31" s="40"/>
-      <c r="I31" s="40">
+      <c r="F31" s="28"/>
+      <c r="G31" s="28"/>
+      <c r="H31" s="28"/>
+      <c r="I31" s="28">
         <f>E31*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>2</v>
       </c>
-      <c r="J31" s="41"/>
+      <c r="J31" s="29"/>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A32" s="40">
+      <c r="A32" s="28">
         <v>79845</v>
       </c>
-      <c r="B32" s="40" t="s">
-        <v>24</v>
-      </c>
-      <c r="C32" s="40">
+      <c r="B32" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C32" s="28">
         <v>20342</v>
       </c>
-      <c r="D32" s="41" t="s">
+      <c r="D32" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="E32" s="42">
-        <v>1</v>
-      </c>
-      <c r="F32" s="40"/>
-      <c r="G32" s="40"/>
-      <c r="H32" s="40"/>
-      <c r="I32" s="40">
+      <c r="E32" s="30">
+        <v>1</v>
+      </c>
+      <c r="F32" s="28"/>
+      <c r="G32" s="28"/>
+      <c r="H32" s="28"/>
+      <c r="I32" s="28">
         <f>E32*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J32" s="41"/>
+      <c r="J32" s="29"/>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A33" s="40">
+      <c r="A33" s="28">
         <v>80705</v>
       </c>
-      <c r="B33" s="40" t="s">
-        <v>24</v>
-      </c>
-      <c r="C33" s="40">
+      <c r="B33" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C33" s="28">
         <v>20343</v>
       </c>
-      <c r="D33" s="41" t="s">
+      <c r="D33" s="29" t="s">
         <v>44</v>
       </c>
-      <c r="E33" s="42">
+      <c r="E33" s="30">
         <v>2</v>
       </c>
-      <c r="F33" s="40"/>
-      <c r="G33" s="40"/>
-      <c r="H33" s="40"/>
-      <c r="I33" s="40">
+      <c r="F33" s="28"/>
+      <c r="G33" s="28"/>
+      <c r="H33" s="28"/>
+      <c r="I33" s="28">
         <f>E33*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>2</v>
       </c>
-      <c r="J33" s="41"/>
+      <c r="J33" s="29"/>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A34" s="40">
+      <c r="A34" s="28">
         <v>79582</v>
       </c>
-      <c r="B34" s="40" t="s">
-        <v>24</v>
-      </c>
-      <c r="C34" s="40">
+      <c r="B34" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C34" s="28">
         <v>26088</v>
       </c>
-      <c r="D34" s="41" t="s">
+      <c r="D34" s="29" t="s">
         <v>45</v>
       </c>
-      <c r="E34" s="42">
+      <c r="E34" s="30">
         <v>4</v>
       </c>
-      <c r="F34" s="40"/>
-      <c r="G34" s="40"/>
-      <c r="H34" s="40"/>
-      <c r="I34" s="40">
+      <c r="F34" s="28"/>
+      <c r="G34" s="28"/>
+      <c r="H34" s="28"/>
+      <c r="I34" s="28">
         <f>E34*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>4</v>
       </c>
-      <c r="J34" s="41"/>
+      <c r="J34" s="29"/>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A35" s="40">
+      <c r="A35" s="28">
         <v>79670</v>
       </c>
-      <c r="B35" s="40" t="s">
-        <v>24</v>
-      </c>
-      <c r="C35" s="40">
+      <c r="B35" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C35" s="28">
         <v>26092</v>
       </c>
-      <c r="D35" s="41" t="s">
+      <c r="D35" s="29" t="s">
         <v>46</v>
       </c>
-      <c r="E35" s="42">
+      <c r="E35" s="30">
         <v>3</v>
       </c>
-      <c r="F35" s="40"/>
-      <c r="G35" s="40"/>
-      <c r="H35" s="40"/>
-      <c r="I35" s="40">
+      <c r="F35" s="28"/>
+      <c r="G35" s="28"/>
+      <c r="H35" s="28"/>
+      <c r="I35" s="28">
         <f>E35*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>3</v>
       </c>
-      <c r="J35" s="41"/>
+      <c r="J35" s="29"/>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A36" s="40">
+      <c r="A36" s="28">
         <v>79583</v>
       </c>
-      <c r="B36" s="40" t="s">
-        <v>24</v>
-      </c>
-      <c r="C36" s="40">
+      <c r="B36" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C36" s="28">
         <v>26093</v>
       </c>
-      <c r="D36" s="41" t="s">
+      <c r="D36" s="29" t="s">
         <v>47</v>
       </c>
-      <c r="E36" s="42">
-        <v>1</v>
-      </c>
-      <c r="F36" s="40"/>
-      <c r="G36" s="40"/>
-      <c r="H36" s="40"/>
-      <c r="I36" s="40">
+      <c r="E36" s="30">
+        <v>1</v>
+      </c>
+      <c r="F36" s="28"/>
+      <c r="G36" s="28"/>
+      <c r="H36" s="28"/>
+      <c r="I36" s="28">
         <f>E36*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J36" s="41"/>
+      <c r="J36" s="29"/>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A37" s="40">
+      <c r="A37" s="28">
         <v>79584</v>
       </c>
-      <c r="B37" s="40" t="s">
-        <v>24</v>
-      </c>
-      <c r="C37" s="40">
+      <c r="B37" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C37" s="28">
         <v>26249</v>
       </c>
-      <c r="D37" s="41" t="s">
+      <c r="D37" s="29" t="s">
         <v>48</v>
       </c>
-      <c r="E37" s="42">
-        <v>1</v>
-      </c>
-      <c r="F37" s="40"/>
-      <c r="G37" s="40"/>
-      <c r="H37" s="40"/>
-      <c r="I37" s="40">
+      <c r="E37" s="30">
+        <v>1</v>
+      </c>
+      <c r="F37" s="28"/>
+      <c r="G37" s="28"/>
+      <c r="H37" s="28"/>
+      <c r="I37" s="28">
         <f>E37*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J37" s="41"/>
+      <c r="J37" s="29"/>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A38" s="40">
+      <c r="A38" s="28">
         <v>79585</v>
       </c>
-      <c r="B38" s="40" t="s">
-        <v>24</v>
-      </c>
-      <c r="C38" s="40">
+      <c r="B38" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C38" s="28">
         <v>26662</v>
       </c>
-      <c r="D38" s="41" t="s">
+      <c r="D38" s="29" t="s">
         <v>49</v>
       </c>
-      <c r="E38" s="42">
-        <v>1</v>
-      </c>
-      <c r="F38" s="40"/>
-      <c r="G38" s="40"/>
-      <c r="H38" s="40"/>
-      <c r="I38" s="40">
+      <c r="E38" s="30">
+        <v>1</v>
+      </c>
+      <c r="F38" s="28"/>
+      <c r="G38" s="28"/>
+      <c r="H38" s="28"/>
+      <c r="I38" s="28">
         <f>E38*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J38" s="41"/>
+      <c r="J38" s="29"/>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A39" s="40">
+      <c r="A39" s="28">
         <v>71525</v>
       </c>
-      <c r="B39" s="40" t="s">
-        <v>24</v>
-      </c>
-      <c r="C39" s="40">
+      <c r="B39" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C39" s="28">
         <v>37310</v>
       </c>
-      <c r="D39" s="41" t="s">
+      <c r="D39" s="29" t="s">
         <v>50</v>
       </c>
-      <c r="E39" s="42">
+      <c r="E39" s="30">
         <v>4</v>
       </c>
-      <c r="F39" s="40"/>
-      <c r="G39" s="40"/>
-      <c r="H39" s="40"/>
-      <c r="I39" s="40">
+      <c r="F39" s="28"/>
+      <c r="G39" s="28"/>
+      <c r="H39" s="28"/>
+      <c r="I39" s="28">
         <f>E39*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>4</v>
       </c>
-      <c r="J39" s="41"/>
+      <c r="J39" s="29"/>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A40" s="40">
+      <c r="A40" s="28">
         <v>79587</v>
       </c>
-      <c r="B40" s="40" t="s">
-        <v>24</v>
-      </c>
-      <c r="C40" s="40">
+      <c r="B40" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C40" s="28">
         <v>37385</v>
       </c>
-      <c r="D40" s="41" t="s">
+      <c r="D40" s="29" t="s">
         <v>51</v>
       </c>
-      <c r="E40" s="42">
+      <c r="E40" s="30">
         <v>2</v>
       </c>
-      <c r="F40" s="40"/>
-      <c r="G40" s="40"/>
-      <c r="H40" s="40"/>
-      <c r="I40" s="40">
+      <c r="F40" s="28"/>
+      <c r="G40" s="28"/>
+      <c r="H40" s="28"/>
+      <c r="I40" s="28">
         <f>E40*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>2</v>
       </c>
-      <c r="J40" s="41"/>
+      <c r="J40" s="29"/>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A41" s="40">
+      <c r="A41" s="28">
         <v>79588</v>
       </c>
-      <c r="B41" s="40" t="s">
-        <v>24</v>
-      </c>
-      <c r="C41" s="40">
+      <c r="B41" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C41" s="28">
         <v>37419</v>
       </c>
-      <c r="D41" s="41" t="s">
+      <c r="D41" s="29" t="s">
         <v>52</v>
       </c>
-      <c r="E41" s="42">
+      <c r="E41" s="30">
         <v>4</v>
       </c>
-      <c r="F41" s="40"/>
-      <c r="G41" s="40"/>
-      <c r="H41" s="40"/>
-      <c r="I41" s="40">
+      <c r="F41" s="28"/>
+      <c r="G41" s="28"/>
+      <c r="H41" s="28"/>
+      <c r="I41" s="28">
         <f>E41*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>4</v>
       </c>
-      <c r="J41" s="41"/>
+      <c r="J41" s="29"/>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A42" s="40">
+      <c r="A42" s="28">
         <v>79589</v>
       </c>
-      <c r="B42" s="40" t="s">
-        <v>24</v>
-      </c>
-      <c r="C42" s="40">
+      <c r="B42" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C42" s="28">
         <v>37438</v>
       </c>
-      <c r="D42" s="41" t="s">
+      <c r="D42" s="29" t="s">
         <v>53</v>
       </c>
-      <c r="E42" s="42">
-        <v>1</v>
-      </c>
-      <c r="F42" s="40"/>
-      <c r="G42" s="40"/>
-      <c r="H42" s="40"/>
-      <c r="I42" s="40">
+      <c r="E42" s="30">
+        <v>1</v>
+      </c>
+      <c r="F42" s="28"/>
+      <c r="G42" s="28"/>
+      <c r="H42" s="28"/>
+      <c r="I42" s="28">
         <f>E42*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J42" s="41"/>
+      <c r="J42" s="29"/>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A43" s="40">
+      <c r="A43" s="28">
         <v>79590</v>
       </c>
-      <c r="B43" s="40" t="s">
-        <v>24</v>
-      </c>
-      <c r="C43" s="40">
+      <c r="B43" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C43" s="28">
         <v>405226</v>
       </c>
-      <c r="D43" s="41" t="s">
+      <c r="D43" s="29" t="s">
         <v>54</v>
       </c>
-      <c r="E43" s="42">
+      <c r="E43" s="30">
         <v>2</v>
       </c>
-      <c r="F43" s="40"/>
-      <c r="G43" s="40"/>
-      <c r="H43" s="40"/>
-      <c r="I43" s="40">
+      <c r="F43" s="28"/>
+      <c r="G43" s="28"/>
+      <c r="H43" s="28"/>
+      <c r="I43" s="28">
         <f>E43*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>2</v>
       </c>
-      <c r="J43" s="41"/>
+      <c r="J43" s="29"/>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A44" s="40">
+      <c r="A44" s="28">
         <v>70806</v>
       </c>
-      <c r="B44" s="40" t="s">
-        <v>24</v>
-      </c>
-      <c r="C44" s="40">
+      <c r="B44" s="28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C44" s="28">
         <v>407752</v>
       </c>
-      <c r="D44" s="41" t="s">
+      <c r="D44" s="29" t="s">
         <v>55</v>
       </c>
-      <c r="E44" s="42">
-        <v>1</v>
-      </c>
-      <c r="F44" s="40"/>
-      <c r="G44" s="40"/>
-      <c r="H44" s="40"/>
-      <c r="I44" s="40">
+      <c r="E44" s="30">
+        <v>1</v>
+      </c>
+      <c r="F44" s="28"/>
+      <c r="G44" s="28"/>
+      <c r="H44" s="28"/>
+      <c r="I44" s="28">
         <f>E44*'[1]OFERTA PARA EL CLIENTE'!$E$17</f>
         <v>1</v>
       </c>
-      <c r="J44" s="41"/>
+      <c r="J44" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="10">

</xml_diff>